<commit_message>
use refrrel code for other
</commit_message>
<xml_diff>
--- a/exports/V2-ambassadors-80pct-15-downloads-2026-10-16.xlsx
+++ b/exports/V2-ambassadors-80pct-15-downloads-2026-10-16.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="172">
   <si>
     <t>#</t>
   </si>
@@ -53,10 +53,7 @@
     <t>Downloads (V2)</t>
   </si>
   <si>
-    <t>Downloads (Oct 2026)</t>
-  </si>
-  <si>
-    <t>Batch A — 6 qualified</t>
+    <t>Batch A — 7 qualified</t>
   </si>
   <si>
     <t>Ramya Aietha</t>
@@ -113,6 +110,21 @@
     <t>27/27</t>
   </si>
   <si>
+    <t>Ryava Bhavana</t>
+  </si>
+  <si>
+    <t>ryavabhavanareddy@gmail.com</t>
+  </si>
+  <si>
+    <t>Engeneering staff college of india</t>
+  </si>
+  <si>
+    <t>DMA16</t>
+  </si>
+  <si>
+    <t>24/27</t>
+  </si>
+  <si>
     <t>Latha Revu</t>
   </si>
   <si>
@@ -227,9 +239,6 @@
     <t>DMB07</t>
   </si>
   <si>
-    <t>24/27</t>
-  </si>
-  <si>
     <t>Bora Chandini</t>
   </si>
   <si>
@@ -488,7 +497,7 @@
     <t/>
   </si>
   <si>
-    <t>Total qualified: 27</t>
+    <t>Total qualified: 28</t>
   </si>
   <si>
     <t>Programme run</t>
@@ -507,9 +516,6 @@
   </si>
   <si>
     <t>&gt;= 15 counted installs recorded in V2 (25 Sept 2026 onward), same as the Downloads column on that table</t>
-  </si>
-  <si>
-    <t>Shown for reference only</t>
   </si>
   <si>
     <t>Ambassadors</t>
@@ -932,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -945,10 +951,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -982,13 +987,10 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -1000,161 +1002,148 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
       <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
       </c>
       <c r="H3" s="1">
         <v>0.81</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
-        <v>32</v>
-      </c>
-      <c r="L3">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
         <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
       </c>
       <c r="H4" s="1">
         <v>0.93</v>
       </c>
       <c r="I4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>30</v>
       </c>
-      <c r="L4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
         <v>28</v>
       </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="1">
-        <v>1</v>
-      </c>
-      <c r="I5" t="s">
-        <v>30</v>
-      </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K5">
         <v>35</v>
       </c>
-      <c r="L5">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
         <v>33</v>
       </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="I6" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="1">
-        <v>1</v>
-      </c>
-      <c r="I6" t="s">
-        <v>30</v>
-      </c>
-      <c r="J6" t="s">
-        <v>20</v>
+      <c r="J6">
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>40</v>
-      </c>
-      <c r="L6">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1168,163 +1157,150 @@
         <v>37</v>
       </c>
       <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K7">
         <v>40</v>
       </c>
-      <c r="L7">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
         <v>40</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>41</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>42</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>16</v>
-      </c>
-      <c r="F8" t="s">
-        <v>17</v>
       </c>
       <c r="G8" t="s">
         <v>43</v>
       </c>
       <c r="H8" s="1">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="1">
         <v>0.85</v>
       </c>
-      <c r="I8" t="s">
-        <v>44</v>
-      </c>
-      <c r="J8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8">
+      <c r="I9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9">
         <v>30</v>
       </c>
-      <c r="L8">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" t="s">
+    </row>
+    <row r="11" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G11" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="1">
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="1">
         <v>0.96</v>
       </c>
-      <c r="I11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J11">
+      <c r="I12" t="s">
+        <v>55</v>
+      </c>
+      <c r="J12">
         <v>6</v>
       </c>
-      <c r="K11">
-        <v>19</v>
-      </c>
-      <c r="L11">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="K12">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>2</v>
-      </c>
-      <c r="B12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" t="s">
-        <v>55</v>
-      </c>
-      <c r="H12" s="1">
-        <v>1</v>
-      </c>
-      <c r="I12" t="s">
-        <v>30</v>
-      </c>
-      <c r="J12" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12">
-        <v>30</v>
-      </c>
-      <c r="L12">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>3</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
@@ -1336,33 +1312,30 @@
         <v>58</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G13" t="s">
         <v>59</v>
       </c>
       <c r="H13" s="1">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>44</v>
-      </c>
-      <c r="J13">
-        <v>2</v>
+        <v>29</v>
+      </c>
+      <c r="J13" t="s">
+        <v>19</v>
       </c>
       <c r="K13">
-        <v>16</v>
-      </c>
-      <c r="L13">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" t="s">
         <v>60</v>
@@ -1374,33 +1347,30 @@
         <v>62</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G14" t="s">
         <v>63</v>
       </c>
       <c r="H14" s="1">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" t="s">
-        <v>20</v>
+        <v>48</v>
+      </c>
+      <c r="J14">
+        <v>2</v>
       </c>
       <c r="K14">
-        <v>30</v>
-      </c>
-      <c r="L14">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
         <v>64</v>
@@ -1412,719 +1382,699 @@
         <v>66</v>
       </c>
       <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" t="s">
         <v>67</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" s="1">
+        <v>0.81</v>
+      </c>
+      <c r="I15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="I16" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" t="s">
+        <v>77</v>
+      </c>
+      <c r="H17" s="1">
+        <v>1</v>
+      </c>
+      <c r="I17" t="s">
+        <v>29</v>
+      </c>
+      <c r="J17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17">
         <v>49</v>
       </c>
-      <c r="G15" t="s">
-        <v>68</v>
-      </c>
-      <c r="H15" s="1">
-        <v>0.89</v>
-      </c>
-      <c r="I15" t="s">
-        <v>69</v>
-      </c>
-      <c r="J15" t="s">
-        <v>20</v>
-      </c>
-      <c r="K15">
-        <v>20</v>
-      </c>
-      <c r="L15">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>6</v>
-      </c>
-      <c r="B16" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-      <c r="I16" t="s">
-        <v>30</v>
-      </c>
-      <c r="J16" t="s">
-        <v>20</v>
-      </c>
-      <c r="K16">
-        <v>49</v>
-      </c>
-      <c r="L16">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>7</v>
       </c>
-      <c r="B17" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" t="s">
-        <v>77</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="B18" t="s">
         <v>78</v>
       </c>
-      <c r="F17" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="C18" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="1">
+      <c r="D18" t="s">
+        <v>80</v>
+      </c>
+      <c r="E18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" t="s">
+        <v>82</v>
+      </c>
+      <c r="H18" s="1">
         <v>0.81</v>
       </c>
-      <c r="I17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17">
-        <v>1</v>
-      </c>
-      <c r="K17">
+      <c r="I18" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
         <v>31</v>
       </c>
-      <c r="L17">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>8</v>
       </c>
-      <c r="B18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" t="s">
-        <v>82</v>
-      </c>
-      <c r="E18" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="B19" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="1">
+      <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" t="s">
+        <v>86</v>
+      </c>
+      <c r="H19" s="1">
         <v>0.93</v>
       </c>
-      <c r="I18" t="s">
-        <v>25</v>
-      </c>
-      <c r="J18" t="s">
-        <v>20</v>
-      </c>
-      <c r="K18">
-        <v>20</v>
-      </c>
-      <c r="L18">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>85</v>
-      </c>
-      <c r="C21" t="s">
-        <v>86</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="I19" t="s">
+        <v>24</v>
+      </c>
+      <c r="J19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E21" t="s">
-        <v>16</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
         <v>88</v>
       </c>
-      <c r="G21" t="s">
+      <c r="C22" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
-        <v>1</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="D22" t="s">
         <v>90</v>
       </c>
-      <c r="J21" t="s">
-        <v>20</v>
-      </c>
-      <c r="K21">
-        <v>28</v>
-      </c>
-      <c r="L21">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" t="s">
+        <v>91</v>
+      </c>
+      <c r="G22" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" t="s">
+        <v>93</v>
+      </c>
+      <c r="J22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>2</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" t="s">
+        <v>95</v>
+      </c>
+      <c r="D23" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="C22" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="G23" t="s">
+        <v>97</v>
+      </c>
+      <c r="H23" s="1">
+        <v>0.91</v>
+      </c>
+      <c r="I23" t="s">
+        <v>98</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="K23">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="1">
+        <v>1</v>
+      </c>
+      <c r="I24" t="s">
         <v>93</v>
       </c>
-      <c r="E22" t="s">
-        <v>16</v>
-      </c>
-      <c r="F22" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" s="1">
-        <v>0.91</v>
-      </c>
-      <c r="I22" t="s">
-        <v>95</v>
-      </c>
-      <c r="J22">
+      <c r="J24" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25" t="s">
+        <v>107</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0.86</v>
+      </c>
+      <c r="I25" t="s">
+        <v>108</v>
+      </c>
+      <c r="J25">
+        <v>1</v>
+      </c>
+      <c r="K25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>110</v>
+      </c>
+      <c r="C28" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" t="s">
+        <v>113</v>
+      </c>
+      <c r="F28" t="s">
+        <v>114</v>
+      </c>
+      <c r="G28" t="s">
+        <v>115</v>
+      </c>
+      <c r="H28" s="1">
+        <v>0.81</v>
+      </c>
+      <c r="I28" t="s">
+        <v>116</v>
+      </c>
+      <c r="J28" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>2</v>
       </c>
-      <c r="K22">
-        <v>44</v>
-      </c>
-      <c r="L22">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="B29" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" t="s">
+        <v>118</v>
+      </c>
+      <c r="D29" t="s">
+        <v>119</v>
+      </c>
+      <c r="E29" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" t="s">
+        <v>114</v>
+      </c>
+      <c r="G29" t="s">
+        <v>120</v>
+      </c>
+      <c r="H29" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="I29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J29" t="s">
+        <v>19</v>
+      </c>
+      <c r="K29">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>3</v>
       </c>
-      <c r="B23" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" t="s">
-        <v>97</v>
-      </c>
-      <c r="D23" t="s">
-        <v>98</v>
-      </c>
-      <c r="E23" t="s">
-        <v>16</v>
-      </c>
-      <c r="F23" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H23" s="1">
-        <v>1</v>
-      </c>
-      <c r="I23" t="s">
-        <v>90</v>
-      </c>
-      <c r="J23" t="s">
-        <v>20</v>
-      </c>
-      <c r="K23">
-        <v>24</v>
-      </c>
-      <c r="L23">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>4</v>
-      </c>
-      <c r="B24" t="s">
-        <v>100</v>
-      </c>
-      <c r="C24" t="s">
-        <v>101</v>
-      </c>
-      <c r="D24" t="s">
-        <v>102</v>
-      </c>
-      <c r="E24" t="s">
-        <v>103</v>
-      </c>
-      <c r="F24" t="s">
-        <v>88</v>
-      </c>
-      <c r="G24" t="s">
-        <v>104</v>
-      </c>
-      <c r="H24" s="1">
-        <v>0.86</v>
-      </c>
-      <c r="I24" t="s">
-        <v>105</v>
-      </c>
-      <c r="J24">
-        <v>1</v>
-      </c>
-      <c r="K24">
-        <v>45</v>
-      </c>
-      <c r="L24">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>1</v>
-      </c>
-      <c r="B27" t="s">
-        <v>107</v>
-      </c>
-      <c r="C27" t="s">
-        <v>108</v>
-      </c>
-      <c r="D27" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" t="s">
-        <v>110</v>
-      </c>
-      <c r="F27" t="s">
-        <v>111</v>
-      </c>
-      <c r="G27" t="s">
-        <v>112</v>
-      </c>
-      <c r="H27" s="1">
-        <v>0.81</v>
-      </c>
-      <c r="I27" t="s">
-        <v>113</v>
-      </c>
-      <c r="J27" t="s">
-        <v>20</v>
-      </c>
-      <c r="K27">
-        <v>40</v>
-      </c>
-      <c r="L27">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>2</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="B30" t="s">
+        <v>122</v>
+      </c>
+      <c r="C30" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" t="s">
+        <v>124</v>
+      </c>
+      <c r="E30" t="s">
+        <v>125</v>
+      </c>
+      <c r="F30" t="s">
         <v>114</v>
       </c>
-      <c r="C28" t="s">
-        <v>115</v>
-      </c>
-      <c r="D28" t="s">
-        <v>116</v>
-      </c>
-      <c r="E28" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" t="s">
-        <v>111</v>
-      </c>
-      <c r="G28" t="s">
-        <v>117</v>
-      </c>
-      <c r="H28" s="1">
+      <c r="G30" t="s">
+        <v>126</v>
+      </c>
+      <c r="H30" s="1">
+        <v>0.95</v>
+      </c>
+      <c r="I30" t="s">
+        <v>127</v>
+      </c>
+      <c r="J30" t="s">
+        <v>19</v>
+      </c>
+      <c r="K30">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" t="s">
+        <v>132</v>
+      </c>
+      <c r="H33" s="1">
         <v>0.9</v>
       </c>
-      <c r="I28" t="s">
-        <v>118</v>
-      </c>
-      <c r="J28" t="s">
-        <v>20</v>
-      </c>
-      <c r="K28">
-        <v>32</v>
-      </c>
-      <c r="L28">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>3</v>
-      </c>
-      <c r="B29" t="s">
-        <v>119</v>
-      </c>
-      <c r="C29" t="s">
-        <v>120</v>
-      </c>
-      <c r="D29" t="s">
-        <v>121</v>
-      </c>
-      <c r="E29" t="s">
-        <v>122</v>
-      </c>
-      <c r="F29" t="s">
-        <v>111</v>
-      </c>
-      <c r="G29" t="s">
-        <v>123</v>
-      </c>
-      <c r="H29" s="1">
-        <v>0.95</v>
-      </c>
-      <c r="I29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J29" t="s">
-        <v>20</v>
-      </c>
-      <c r="K29">
-        <v>25</v>
-      </c>
-      <c r="L29">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>1</v>
-      </c>
-      <c r="B32" t="s">
-        <v>126</v>
-      </c>
-      <c r="C32" t="s">
-        <v>127</v>
-      </c>
-      <c r="D32" t="s">
-        <v>20</v>
-      </c>
-      <c r="E32" t="s">
-        <v>16</v>
-      </c>
-      <c r="F32" t="s">
-        <v>128</v>
-      </c>
-      <c r="G32" t="s">
-        <v>129</v>
-      </c>
-      <c r="H32" s="1">
-        <v>0.9</v>
-      </c>
-      <c r="I32" t="s">
-        <v>130</v>
-      </c>
-      <c r="J32">
-        <v>1</v>
-      </c>
-      <c r="K32">
-        <v>31</v>
-      </c>
-      <c r="L32">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>2</v>
-      </c>
-      <c r="B33" t="s">
-        <v>131</v>
-      </c>
-      <c r="C33" t="s">
-        <v>132</v>
-      </c>
-      <c r="D33" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" t="s">
-        <v>16</v>
-      </c>
-      <c r="F33" t="s">
-        <v>128</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="I33" t="s">
         <v>133</v>
       </c>
-      <c r="H33" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="I33" t="s">
-        <v>134</v>
-      </c>
-      <c r="J33" t="s">
-        <v>20</v>
+      <c r="J33">
+        <v>1</v>
       </c>
       <c r="K33">
         <v>31</v>
       </c>
-      <c r="L33">
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>2</v>
+      </c>
+      <c r="B34" t="s">
+        <v>134</v>
+      </c>
+      <c r="C34" t="s">
+        <v>135</v>
+      </c>
+      <c r="D34" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" t="s">
+        <v>136</v>
+      </c>
+      <c r="H34" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="I34" t="s">
+        <v>137</v>
+      </c>
+      <c r="J34" t="s">
+        <v>19</v>
+      </c>
+      <c r="K34">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>138</v>
+      </c>
+      <c r="C35" t="s">
+        <v>139</v>
+      </c>
+      <c r="D35" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" t="s">
+        <v>15</v>
+      </c>
+      <c r="F35" t="s">
+        <v>131</v>
+      </c>
+      <c r="G35" t="s">
+        <v>140</v>
+      </c>
+      <c r="H35" s="1">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>141</v>
+      </c>
+      <c r="J35" t="s">
+        <v>19</v>
+      </c>
+      <c r="K35">
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>3</v>
-      </c>
-      <c r="B34" t="s">
-        <v>135</v>
-      </c>
-      <c r="C34" t="s">
-        <v>136</v>
-      </c>
-      <c r="D34" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" t="s">
-        <v>16</v>
-      </c>
-      <c r="F34" t="s">
-        <v>128</v>
-      </c>
-      <c r="G34" t="s">
+    <row r="37" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" t="s">
+        <v>143</v>
+      </c>
+      <c r="C38" t="s">
+        <v>144</v>
+      </c>
+      <c r="D38" t="s">
+        <v>145</v>
+      </c>
+      <c r="E38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" t="s">
+        <v>146</v>
+      </c>
+      <c r="G38" t="s">
+        <v>147</v>
+      </c>
+      <c r="H38" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="I38" t="s">
         <v>137</v>
       </c>
-      <c r="H34" s="1">
-        <v>1</v>
-      </c>
-      <c r="I34" t="s">
-        <v>138</v>
-      </c>
-      <c r="J34" t="s">
-        <v>20</v>
-      </c>
-      <c r="K34">
-        <v>30</v>
-      </c>
-      <c r="L34">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>1</v>
-      </c>
-      <c r="B37" t="s">
-        <v>140</v>
-      </c>
-      <c r="C37" t="s">
-        <v>141</v>
-      </c>
-      <c r="D37" t="s">
-        <v>142</v>
-      </c>
-      <c r="E37" t="s">
-        <v>16</v>
-      </c>
-      <c r="F37" t="s">
-        <v>143</v>
-      </c>
-      <c r="G37" t="s">
-        <v>144</v>
-      </c>
-      <c r="H37" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="I37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J37">
-        <v>3</v>
-      </c>
-      <c r="K37">
+      <c r="J38">
+        <v>4</v>
+      </c>
+      <c r="K38">
         <v>29</v>
       </c>
-      <c r="L37">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38">
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>2</v>
       </c>
-      <c r="B38" t="s">
-        <v>145</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="B39" t="s">
+        <v>148</v>
+      </c>
+      <c r="C39" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" t="s">
         <v>146</v>
       </c>
-      <c r="D38" t="s">
-        <v>147</v>
-      </c>
-      <c r="E38" t="s">
-        <v>148</v>
-      </c>
-      <c r="F38" t="s">
-        <v>143</v>
-      </c>
-      <c r="G38" t="s">
-        <v>149</v>
-      </c>
-      <c r="H38" s="1">
-        <v>0.95</v>
-      </c>
-      <c r="I38" t="s">
-        <v>150</v>
-      </c>
-      <c r="J38">
-        <v>1</v>
-      </c>
-      <c r="K38">
-        <v>23</v>
-      </c>
-      <c r="L38">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>3</v>
-      </c>
-      <c r="B39" t="s">
-        <v>151</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="G39" t="s">
         <v>152</v>
-      </c>
-      <c r="D39" t="s">
-        <v>153</v>
-      </c>
-      <c r="E39" t="s">
-        <v>16</v>
-      </c>
-      <c r="F39" t="s">
-        <v>143</v>
-      </c>
-      <c r="G39" t="s">
-        <v>154</v>
       </c>
       <c r="H39" s="1">
         <v>0.95</v>
       </c>
       <c r="I39" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J39">
         <v>1</v>
       </c>
       <c r="K39">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>3</v>
+      </c>
+      <c r="B40" t="s">
+        <v>154</v>
+      </c>
+      <c r="C40" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" t="s">
+        <v>156</v>
+      </c>
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" t="s">
+        <v>146</v>
+      </c>
+      <c r="G40" t="s">
+        <v>157</v>
+      </c>
+      <c r="H40" s="1">
+        <v>0.95</v>
+      </c>
+      <c r="I40" t="s">
+        <v>153</v>
+      </c>
+      <c r="J40">
+        <v>1</v>
+      </c>
+      <c r="K40">
         <v>38</v>
       </c>
-      <c r="L39">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="H41" s="7"/>
+    </row>
+    <row r="42" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H42" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A10:L10"/>
-    <mergeCell ref="A20:L20"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="A36:L36"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A27:K27"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A37:K37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2133,7 +2083,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2146,10 +2096,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2183,163 +2132,148 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
       </c>
       <c r="H2" s="1">
         <v>0.81</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K2">
-        <v>32</v>
-      </c>
-      <c r="L2">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
         <v>23</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>24</v>
       </c>
       <c r="H3" s="1">
         <v>0.93</v>
       </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
         <v>30</v>
       </c>
-      <c r="L3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="1">
-        <v>1</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>35</v>
       </c>
-      <c r="L4">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="I5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="1">
-        <v>1</v>
-      </c>
-      <c r="I5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" t="s">
-        <v>20</v>
+      <c r="J5">
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>40</v>
-      </c>
-      <c r="L5">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2353,70 +2287,99 @@
         <v>37</v>
       </c>
       <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>39</v>
-      </c>
       <c r="H6" s="1">
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K6">
         <v>40</v>
       </c>
-      <c r="L6">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
         <v>40</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>17</v>
       </c>
       <c r="G7" t="s">
         <v>43</v>
       </c>
       <c r="H7" s="1">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="1">
         <v>0.85</v>
       </c>
-      <c r="I7" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" t="s">
-        <v>20</v>
-      </c>
-      <c r="K7">
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8">
         <v>30</v>
       </c>
-      <c r="L7">
-        <v>29</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2424,7 +2387,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2437,10 +2400,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2474,37 +2436,34 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H2" s="1">
         <v>0.96</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J2">
         <v>6</v>
@@ -2512,75 +2471,69 @@
       <c r="K2">
         <v>19</v>
       </c>
-      <c r="L2">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>53</v>
       </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>49</v>
-      </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H3" s="1">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
         <v>30</v>
       </c>
-      <c r="L3">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H4" s="1">
         <v>0.85</v>
       </c>
       <c r="I4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="J4">
         <v>2</v>
@@ -2588,151 +2541,139 @@
       <c r="K4">
         <v>16</v>
       </c>
-      <c r="L4">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H5" s="1">
         <v>0.81</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K5">
         <v>30</v>
       </c>
-      <c r="L5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H6" s="1">
         <v>0.89</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K6">
         <v>20</v>
       </c>
-      <c r="L6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K7">
         <v>49</v>
       </c>
-      <c r="L7">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H8" s="1">
         <v>0.81</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -2740,50 +2681,44 @@
       <c r="K8">
         <v>31</v>
       </c>
-      <c r="L8">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H9" s="1">
         <v>0.93</v>
       </c>
       <c r="I9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9">
-        <v>20</v>
-      </c>
-      <c r="L9">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2791,7 +2726,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2804,10 +2739,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2841,151 +2775,139 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H2" s="1">
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K2">
-        <v>28</v>
-      </c>
-      <c r="L2">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>91</v>
       </c>
-      <c r="C3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>88</v>
-      </c>
       <c r="G3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H3" s="1">
         <v>0.91</v>
       </c>
       <c r="I3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>44</v>
-      </c>
-      <c r="L3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>24</v>
       </c>
-      <c r="L4">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H5" s="1">
         <v>0.86</v>
       </c>
       <c r="I5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -2993,12 +2915,9 @@
       <c r="K5">
         <v>45</v>
       </c>
-      <c r="L5">
-        <v>39</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3006,7 +2925,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -3019,10 +2938,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3056,126 +2974,114 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H2" s="1">
         <v>0.81</v>
       </c>
       <c r="I2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K2">
         <v>40</v>
       </c>
-      <c r="L2">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>114</v>
       </c>
-      <c r="C3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>111</v>
-      </c>
       <c r="G3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H3" s="1">
         <v>0.9</v>
       </c>
       <c r="I3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
         <v>32</v>
       </c>
-      <c r="L3">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H4" s="1">
         <v>0.95</v>
       </c>
       <c r="I4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
-        <v>25</v>
-      </c>
-      <c r="L4">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3183,7 +3089,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -3196,10 +3102,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3233,37 +3138,34 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="G2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="H2" s="1">
         <v>0.9</v>
       </c>
       <c r="I2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -3271,88 +3173,79 @@
       <c r="K2">
         <v>31</v>
       </c>
-      <c r="L2">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>131</v>
       </c>
-      <c r="C3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>128</v>
-      </c>
       <c r="G3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H3" s="1">
         <v>0.8</v>
       </c>
       <c r="I3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
         <v>31</v>
       </c>
-      <c r="L3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="G4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>30</v>
       </c>
-      <c r="L4">
-        <v>9</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3360,7 +3253,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -3373,10 +3266,9 @@
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3410,75 +3302,69 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H2" s="1">
         <v>0.8</v>
       </c>
       <c r="I2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2">
         <v>29</v>
       </c>
-      <c r="L2">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F3" t="s">
         <v>146</v>
       </c>
-      <c r="D3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F3" t="s">
-        <v>143</v>
-      </c>
       <c r="G3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="H3" s="1">
         <v>0.95</v>
       </c>
       <c r="I3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -3486,37 +3372,34 @@
       <c r="K3">
         <v>23</v>
       </c>
-      <c r="L3">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H4" s="1">
         <v>0.95</v>
       </c>
       <c r="I4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -3524,12 +3407,9 @@
       <c r="K4">
         <v>38</v>
       </c>
-      <c r="L4">
-        <v>38</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3537,7 +3417,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" style="6" customWidth="1"/>
@@ -3546,95 +3426,95 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>11</v>
+        <v>166</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B5" t="s">
-        <v>165</v>
+        <v>168</v>
+      </c>
+      <c r="B5">
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B7" t="s">
-        <v>168</v>
+        <v>169</v>
+      </c>
+      <c r="B6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B8" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="B9" t="s">
-        <v>155</v>
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="B10">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="B11">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -3642,17 +3522,9 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="B14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B15">
         <v>3</v>
       </c>
     </row>

</xml_diff>